<commit_message>
updated and added png extraction of dxfs file
</commit_message>
<xml_diff>
--- a/Solidworks/DXFs-Sorter/example/DXFs List.xlsx
+++ b/Solidworks/DXFs-Sorter/example/DXFs List.xlsx
@@ -1,78 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Solidworks\missed dxfs\New folder\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF97154-2E87-4334-922A-78D1E0E8DB64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{90AC5FBF-3BB6-4242-BD24-9D969A2338EB}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
-  <si>
-    <t>ITEM NO.</t>
-  </si>
-  <si>
-    <t>PART NUMBER</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Sheet Metal Thickness</t>
-  </si>
-  <si>
-    <t>Bends</t>
-  </si>
-  <si>
-    <t>QTY.</t>
-  </si>
-  <si>
-    <t>Sheet</t>
-  </si>
-  <si>
-    <t>Tension Plate_wd02</t>
-  </si>
-  <si>
-    <t>web1 side sheet structural support 2_wd02</t>
-  </si>
-  <si>
-    <t>Transfer sheet web1-web2 mounting bracket_wd02</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -106,31 +61,176 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="171450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -429,99 +529,129 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BACC012-9938-407F-A8F2-9151A23F28F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="43.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col width="43.6640625" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
+    <col width="10.21875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="19.21875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="5.88671875" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="4.88671875" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="20.71428571428572" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ITEM NO.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PART NUMBER</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sheet Metal Thickness</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Bends</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>QTY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="75" customHeight="1">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Tension Plate_wd02</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="3" ht="75" customHeight="1">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>web1 side sheet structural support 2_wd02</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="1">
-        <v>5</v>
-      </c>
-      <c r="E2" s="1">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Transfer sheet web1-web2 mounting bracket_wd02</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="1">
-        <v>5</v>
-      </c>
-      <c r="E3" s="1">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="1">
-        <v>3</v>
-      </c>
-      <c r="E4" s="1">
-        <v>0</v>
-      </c>
-      <c r="F4" s="1">
+      <c r="F4" s="1" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
get row to insert pngs
</commit_message>
<xml_diff>
--- a/Solidworks/DXFs-Sorter/example/DXFs List.xlsx
+++ b/Solidworks/DXFs-Sorter/example/DXFs List.xlsx
@@ -220,6 +220,2246 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="581025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="257175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1152525" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="552450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="523875" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1352550" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="657225" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="638175" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="171450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="657225" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="923925" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="523875" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1419225" cy="447675"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="942975"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="581025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="257175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1152525" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="552450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="523875" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1352550" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="657225" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="638175" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="171450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="657225" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="923925" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="523875" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1419225" cy="447675"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="942975"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="581025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="257175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId46"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1152525" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="552450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId50"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId51"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="523875" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId52"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1352550" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId53"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="657225" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId54"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="638175" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId55"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="171450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId56"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId57"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="657225" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId58"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="923925" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId59"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="523875" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="60" name="Image 60" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId60"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1419225" cy="447675"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="61" name="Image 61" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId61"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="62" name="Image 62" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId62"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="942975"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="63" name="Image 63" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId63"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="581025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId64"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="257175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId65"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId66"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="67" name="Image 67" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId67"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="68" name="Image 68" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId68"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1152525" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="69" name="Image 69" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId69"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="552450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="70" name="Image 70" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId70"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="962025" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="71" name="Image 71" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId71"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="523875" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="72" name="Image 72" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId72"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1352550" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="73" name="Image 73" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId73"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="657225" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="74" name="Image 74" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId74"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="638175" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="75" name="Image 75" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId75"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="171450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="76" name="Image 76" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId76"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="77" name="Image 77" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId77"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="657225" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="78" name="Image 78" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId78"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="923925" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="79" name="Image 79" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId79"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="523875" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="80" name="Image 80" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId80"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1419225" cy="447675"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="81" name="Image 81" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId81"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="238125" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="82" name="Image 82" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId82"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="942975"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="83" name="Image 83" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId83"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -539,10 +2779,12 @@
   <cols>
     <col width="43.6640625" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
     <col width="10.21875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="19.21875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="20.71428571428572" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="5.88671875" bestFit="1" customWidth="1" min="5" max="5"/>
     <col width="4.88671875" bestFit="1" customWidth="1" min="6" max="6"/>
     <col width="20.71428571428572" customWidth="1" min="7" max="7"/>
+    <col width="20.71428571428572" customWidth="1" min="8" max="8"/>
+    <col width="20.71428571428572" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="75" customHeight="1">
@@ -625,7 +2867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="75" customHeight="1">
       <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
@@ -649,6 +2891,22 @@
         <v>1</v>
       </c>
     </row>
+    <row r="5" ht="75" customHeight="1"/>
+    <row r="6" ht="75" customHeight="1"/>
+    <row r="7" ht="75" customHeight="1"/>
+    <row r="8" ht="75" customHeight="1"/>
+    <row r="9" ht="75" customHeight="1"/>
+    <row r="10" ht="75" customHeight="1"/>
+    <row r="11" ht="75" customHeight="1"/>
+    <row r="12" ht="75" customHeight="1"/>
+    <row r="13" ht="75" customHeight="1"/>
+    <row r="14" ht="75" customHeight="1"/>
+    <row r="15" ht="75" customHeight="1"/>
+    <row r="16" ht="75" customHeight="1"/>
+    <row r="17" ht="75" customHeight="1"/>
+    <row r="18" ht="75" customHeight="1"/>
+    <row r="19" ht="75" customHeight="1"/>
+    <row r="20" ht="75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>